<commit_message>
Update BTC price log - 2026-09-13 02:49 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E318"/>
+  <dimension ref="A1:E319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7100,6 +7100,27 @@
         <v>0.06</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>02:49:29</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>77291</v>
+      </c>
+      <c r="D319" t="n">
+        <v>7389029</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-13 13:06 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E319"/>
+  <dimension ref="A1:E320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7121,6 +7121,27 @@
         <v>0.06</v>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>13:06:14</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>76704</v>
+      </c>
+      <c r="D320" t="n">
+        <v>7332972</v>
+      </c>
+      <c r="E320" t="n">
+        <v>-0.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-13 17:11 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E320"/>
+  <dimension ref="A1:E321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7142,6 +7142,27 @@
         <v>-0.79</v>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>17:11:53</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>77322</v>
+      </c>
+      <c r="D321" t="n">
+        <v>7392023</v>
+      </c>
+      <c r="E321" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-13 20:12 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7163,6 +7163,27 @@
         <v>-0.07000000000000001</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>20:12:01</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>77250</v>
+      </c>
+      <c r="D322" t="n">
+        <v>7381682</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-13 22:48 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E322"/>
+  <dimension ref="A1:E323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7184,6 +7184,27 @@
         <v>0.11</v>
       </c>
     </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>22:48:36</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>76732</v>
+      </c>
+      <c r="D323" t="n">
+        <v>7332655</v>
+      </c>
+      <c r="E323" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-14 00:38 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E323"/>
+  <dimension ref="A1:E324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7205,6 +7205,27 @@
         <v>-0.6</v>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>00:38:39</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>76702</v>
+      </c>
+      <c r="D324" t="n">
+        <v>7248614</v>
+      </c>
+      <c r="E324" t="n">
+        <v>-0.72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-14 05:42 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E324"/>
+  <dimension ref="A1:E325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7226,6 +7226,27 @@
         <v>-0.72</v>
       </c>
     </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>05:42:18</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>77580</v>
+      </c>
+      <c r="D325" t="n">
+        <v>7422967</v>
+      </c>
+      <c r="E325" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-14 11:35 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7247,6 +7247,27 @@
         <v>0.39</v>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>11:35:56</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>77736</v>
+      </c>
+      <c r="D326" t="n">
+        <v>7444126</v>
+      </c>
+      <c r="E326" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-14 17:31 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E326"/>
+  <dimension ref="A1:E327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7268,6 +7268,27 @@
         <v>1.38</v>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>17:31:14</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>78852</v>
+      </c>
+      <c r="D327" t="n">
+        <v>7550516</v>
+      </c>
+      <c r="E327" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-14 21:21 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E327"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7289,6 +7289,27 @@
         <v>2.04</v>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>21:21:20</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>78922</v>
+      </c>
+      <c r="D328" t="n">
+        <v>7563480</v>
+      </c>
+      <c r="E328" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 00:11 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7310,6 +7310,27 @@
         <v>2.02</v>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>00:11:50</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>78218</v>
+      </c>
+      <c r="D329" t="n">
+        <v>7496073</v>
+      </c>
+      <c r="E329" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 05:43 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E329"/>
+  <dimension ref="A1:E330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7331,6 +7331,27 @@
         <v>1.72</v>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>05:43:26</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>77427</v>
+      </c>
+      <c r="D330" t="n">
+        <v>7423154</v>
+      </c>
+      <c r="E330" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 10:55 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E330"/>
+  <dimension ref="A1:E331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7352,6 +7352,27 @@
         <v>-0.11</v>
       </c>
     </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>10:55:49</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>77019</v>
+      </c>
+      <c r="D331" t="n">
+        <v>7383661</v>
+      </c>
+      <c r="E331" t="n">
+        <v>-1.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 15:25 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E331"/>
+  <dimension ref="A1:E332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7373,6 +7373,27 @@
         <v>-1.13</v>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>15:25:44</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>76084</v>
+      </c>
+      <c r="D332" t="n">
+        <v>7299306</v>
+      </c>
+      <c r="E332" t="n">
+        <v>-3.07</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 19:28 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E332"/>
+  <dimension ref="A1:E333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7394,6 +7394,27 @@
         <v>-3.07</v>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>19:28:29</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>76079</v>
+      </c>
+      <c r="D333" t="n">
+        <v>7300719</v>
+      </c>
+      <c r="E333" t="n">
+        <v>-3.92</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-15 22:40 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E333"/>
+  <dimension ref="A1:E334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7415,6 +7415,27 @@
         <v>-3.92</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>22:40:07</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>75574</v>
+      </c>
+      <c r="D334" t="n">
+        <v>7254557</v>
+      </c>
+      <c r="E334" t="n">
+        <v>-3.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BTC price log - 2026-09-16 01:00 UTC
</commit_message>
<xml_diff>
--- a/bitcoin_price_log.xlsx
+++ b/bitcoin_price_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E334"/>
+  <dimension ref="A1:E335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7436,6 +7436,27 @@
         <v>-3.85</v>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>01:00:22</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>75730</v>
+      </c>
+      <c r="D335" t="n">
+        <v>7269599</v>
+      </c>
+      <c r="E335" t="n">
+        <v>-2.84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>